<commit_message>
chore(ci): align GitHub Actions workflow name, job names, and artifact names with the reference visual image
</commit_message>
<xml_diff>
--- a/appium/Appium_E2E_Test_Report_Traverse.xlsx
+++ b/appium/Appium_E2E_Test_Report_Traverse.xlsx
@@ -570,7 +570,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Automated &amp; Simulated Mobile E2E Validation Summary — Generated 2026-06-17 14:54:56</t>
+          <t>Automated &amp; Simulated Mobile E2E Validation Summary — Generated 2026-06-18 09:28:54</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="H3" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="H31" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="H33" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="H35" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="H36" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="H40" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="H51" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="H53" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="H54" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="H57" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="H58" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="H59" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="H60" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="H61" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="H63" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="H64" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="H65" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
       </c>
       <c r="H66" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="H67" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3709,7 @@
       </c>
       <c r="H68" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="H69" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="H70" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="H71" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3877,7 @@
       </c>
       <c r="H72" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="H73" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="H75" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4045,7 @@
       </c>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="H77" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="H79" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="H80" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="H81" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="H83" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="H84" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="H85" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="H86" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="H87" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="H88" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="H89" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="H90" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4675,7 @@
       </c>
       <c r="H91" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="H92" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="H93" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="H94" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="H95" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4885,7 +4885,7 @@
       </c>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="H97" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -4969,7 +4969,7 @@
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="H99" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="H101" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -5137,7 +5137,7 @@
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="H103" s="18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>

</xml_diff>